<commit_message>
feat(sprint1): Complete Sprint 1 - Mobile app + Backend fixes + Cleanup
MOBILE APP (NEW):
- ✅ 9 screens with Expo Router
- ✅ All 7 User Stories implemented
- ✅ Medical History bonus feature
- ✅ DateTimePicker integration
- ✅ API integration with auth
- ✅ Pull-to-refresh, search, filter
- ✅ Empty states with CTA buttons
- ✅ Debug token screen

BACKEND FIXES:
- ✅ DoctorsController null-safe fixes
- ✅ Consistent PublicId/FullName format
- ✅ Fixed 500 error on doctor detail

BUG FIXES:
- ✅ Appointments interface compatibility
- ✅ Medical History interface updated
- ✅ Enhanced error handling (401/404)
- ✅ Removed unnecessary alerts

SCRIPTS ADDED:
- ✅ start-dev.ps1 (dev server)
- ✅ install-datetimepicker.ps1
- ✅ restart-backend.ps1
- ✅ test-mobile-connection.ps1
- ✅ update-ip.ps1
- ✅ cleanup-project.ps1

DOCUMENTATION:
- ✅ SPRINT1_COMPLETION_REPORT.md
- ✅ TESTING_GUIDE.md
- ✅ README_SPRINT1.md
- ✅ Cleaned up 33 temp/debug files

Sprint 1: 12/12 tasks (100%)
Ready for demo and Sprint 2!
</commit_message>
<xml_diff>
--- a/Docs/Nhom8_HeThongPhongKham_Ver02.xlsx
+++ b/Docs/Nhom8_HeThongPhongKham_Ver02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2.CNPMNangCao\LyThuyet\Tuan04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638772F5-CE95-4125-85E8-E55EC381D727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1766746C-E740-4530-A051-14EF5343604A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="798" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="798" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Information" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="136">
   <si>
     <t>I. Requirements</t>
   </si>
@@ -426,6 +426,24 @@
   </si>
   <si>
     <t>Tra cứu thông tin đặt lịch khám của khách hàng</t>
+  </si>
+  <si>
+    <t>17/9/2025</t>
+  </si>
+  <si>
+    <t>30/9/2025</t>
+  </si>
+  <si>
+    <t>26/9/2025</t>
+  </si>
+  <si>
+    <t>27/9/2025</t>
+  </si>
+  <si>
+    <t>28/9/2025</t>
+  </si>
+  <si>
+    <t>29/9/2025</t>
   </si>
 </sst>
 </file>
@@ -489,7 +507,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +556,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="24">
     <border>
@@ -811,7 +835,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -997,7 +1021,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -2367,7 +2393,9 @@
       <c r="D4" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="E4" s="44"/>
+      <c r="E4" s="44" t="s">
+        <v>130</v>
+      </c>
       <c r="F4" s="41"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -2484,7 +2512,7 @@
       <c r="C6" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="37">
+      <c r="D6" s="78">
         <v>2</v>
       </c>
     </row>
@@ -2493,10 +2521,10 @@
         <f>B6+1</f>
         <v>2</v>
       </c>
-      <c r="C7" s="77" t="s">
+      <c r="C7" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="77">
         <v>2</v>
       </c>
       <c r="H7" s="11"/>
@@ -2509,7 +2537,7 @@
       <c r="C8" s="45" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="77">
         <v>2</v>
       </c>
       <c r="H8" s="11"/>
@@ -2522,7 +2550,7 @@
       <c r="C9" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="77">
         <v>2</v>
       </c>
       <c r="H9" s="11"/>
@@ -2587,7 +2615,7 @@
       <c r="C14" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="77">
         <v>2</v>
       </c>
     </row>
@@ -2599,7 +2627,7 @@
       <c r="C15" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="77">
         <v>4</v>
       </c>
     </row>
@@ -2611,7 +2639,7 @@
       <c r="C16" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="77">
         <v>2</v>
       </c>
     </row>
@@ -3095,7 +3123,7 @@
       <c r="F6" s="73"/>
       <c r="G6" s="73"/>
       <c r="H6" s="73"/>
-      <c r="I6" s="73"/>
+      <c r="I6" s="74"/>
       <c r="J6" s="73"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
@@ -3111,18 +3139,28 @@
       <c r="D7" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
+      <c r="E7" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H7" s="79" t="s">
+        <v>132</v>
+      </c>
+      <c r="I7" s="4">
+        <v>2</v>
+      </c>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="31">
         <v>2</v>
       </c>
-      <c r="B8" s="77" t="s">
+      <c r="B8" t="s">
         <v>124</v>
       </c>
       <c r="C8" s="33">
@@ -3131,12 +3169,22 @@
       <c r="D8" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
+      <c r="E8" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H8" s="79" t="s">
+        <v>133</v>
+      </c>
+      <c r="I8" s="4">
+        <v>2</v>
+      </c>
+      <c r="J8" s="48"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="31">
@@ -3151,12 +3199,22 @@
       <c r="D9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
+      <c r="E9" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="H9" s="79" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="4">
+        <v>2</v>
+      </c>
+      <c r="J9" s="48"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="31">
@@ -3171,12 +3229,22 @@
       <c r="D10" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
+      <c r="E10" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" s="79" t="s">
+        <v>134</v>
+      </c>
+      <c r="I10" s="4">
+        <v>4</v>
+      </c>
+      <c r="J10" s="48"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="31">
@@ -3191,12 +3259,22 @@
       <c r="D11" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
+      <c r="E11" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="H11" s="79" t="s">
+        <v>131</v>
+      </c>
+      <c r="I11" s="4">
+        <v>2</v>
+      </c>
+      <c r="J11" s="48"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="31">
@@ -3211,12 +3289,22 @@
       <c r="D12" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
+      <c r="E12" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="H12" s="79" t="s">
+        <v>134</v>
+      </c>
+      <c r="I12" s="4">
+        <v>2</v>
+      </c>
+      <c r="J12" s="48"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="31">
@@ -3231,12 +3319,22 @@
       <c r="D13" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
+      <c r="E13" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="H13" s="79" t="s">
+        <v>135</v>
+      </c>
+      <c r="I13" s="4">
+        <v>2</v>
+      </c>
+      <c r="J13" s="48"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="72"/>

</xml_diff>

<commit_message>
feat: Implement walk-in patients, fix API error handling, and reschedule functionality
- Backend: Add WalkInPatient model and CRUD endpoints
- Backend: Fix GetAppointments to support both Patient and WalkInPatient
- Backend: Add reschedule appointment endpoint for reception
- Frontend: Enhance API error handling with safe JSON parsing
- Frontend: Fix reschedule button event listener issues
- Frontend: Add auto-logout on 401 unauthorized
- Mobile: Fix network errors and API integration
- Docs: Add SQL migration scripts for walk-in patients
- Docs: Update Sprint 2 and Sprint 3 documentation
</commit_message>
<xml_diff>
--- a/Docs/Nhom8_HeThongPhongKham_Ver02.xlsx
+++ b/Docs/Nhom8_HeThongPhongKham_Ver02.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2.CNPMNangCao\LyThuyet\Tuan04\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2.CNPMNangCao\LyThuyet\Tuan07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1766746C-E740-4530-A051-14EF5343604A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4CA6BE-6BB1-4828-BC8C-7B76A9BFCDF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="798" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="141">
   <si>
     <t>I. Requirements</t>
   </si>
@@ -444,6 +444,21 @@
   </si>
   <si>
     <t>29/9/2025</t>
+  </si>
+  <si>
+    <t>410/2025</t>
+  </si>
+  <si>
+    <t>15/10/2025</t>
+  </si>
+  <si>
+    <t>13/10/2025</t>
+  </si>
+  <si>
+    <t>14/10/2025</t>
+  </si>
+  <si>
+    <t>21/10/2025</t>
   </si>
 </sst>
 </file>
@@ -507,7 +522,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -559,6 +574,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -835,7 +862,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -949,6 +976,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
@@ -1021,9 +1065,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -1099,9 +1140,9 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FFFFD9D9"/>
       <color rgb="FF00B050"/>
       <color rgb="FFCCFFCC"/>
-      <color rgb="FFFFD9D9"/>
       <color rgb="FFFF6D6D"/>
       <color rgb="FFFFFFCC"/>
     </mruColors>
@@ -1448,836 +1489,836 @@
       </c>
     </row>
     <row r="3" spans="2:14" ht="18" x14ac:dyDescent="0.2">
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="73" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-      <c r="L3" s="63"/>
-      <c r="M3" s="64"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="75"/>
     </row>
     <row r="4" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="64" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="55"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="66"/>
       <c r="N4" s="29"/>
     </row>
     <row r="5" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="55"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="66"/>
       <c r="N5" s="29"/>
     </row>
     <row r="6" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="55"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="65"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="65"/>
+      <c r="M6" s="66"/>
       <c r="N6" s="29"/>
     </row>
     <row r="7" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="64" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="54"/>
-      <c r="L7" s="54"/>
-      <c r="M7" s="55"/>
+      <c r="C7" s="65"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="66"/>
       <c r="N7" s="29"/>
     </row>
     <row r="8" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="64" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="54"/>
-      <c r="L8" s="54"/>
-      <c r="M8" s="55"/>
+      <c r="C8" s="65"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="65"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
+      <c r="I8" s="65"/>
+      <c r="J8" s="65"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="65"/>
+      <c r="M8" s="66"/>
       <c r="N8" s="29"/>
     </row>
     <row r="9" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="64" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="54"/>
-      <c r="K9" s="54"/>
-      <c r="L9" s="54"/>
-      <c r="M9" s="55"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
+      <c r="I9" s="65"/>
+      <c r="J9" s="65"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="65"/>
+      <c r="M9" s="66"/>
       <c r="N9" s="29"/>
     </row>
     <row r="10" spans="2:14" ht="18" x14ac:dyDescent="0.2">
-      <c r="B10" s="65" t="s">
+      <c r="B10" s="76" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="66"/>
-      <c r="I10" s="66"/>
-      <c r="J10" s="66"/>
-      <c r="K10" s="66"/>
-      <c r="L10" s="66"/>
-      <c r="M10" s="67"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="77"/>
+      <c r="J10" s="77"/>
+      <c r="K10" s="77"/>
+      <c r="L10" s="77"/>
+      <c r="M10" s="78"/>
       <c r="N10" s="29"/>
     </row>
     <row r="11" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="67" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="57"/>
-      <c r="F11" s="57"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
-      <c r="I11" s="57"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="58"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
+      <c r="E11" s="68"/>
+      <c r="F11" s="68"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="68"/>
+      <c r="I11" s="68"/>
+      <c r="J11" s="68"/>
+      <c r="K11" s="68"/>
+      <c r="L11" s="68"/>
+      <c r="M11" s="69"/>
       <c r="N11" s="29"/>
     </row>
     <row r="12" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="64" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="54"/>
-      <c r="K12" s="54"/>
-      <c r="L12" s="54"/>
-      <c r="M12" s="55"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="65"/>
+      <c r="K12" s="65"/>
+      <c r="L12" s="65"/>
+      <c r="M12" s="66"/>
       <c r="N12" s="29"/>
     </row>
     <row r="13" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="54"/>
-      <c r="K13" s="54"/>
-      <c r="L13" s="54"/>
-      <c r="M13" s="55"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="65"/>
+      <c r="I13" s="65"/>
+      <c r="J13" s="65"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="65"/>
+      <c r="M13" s="66"/>
       <c r="N13" s="29"/>
     </row>
     <row r="14" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="55"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="65"/>
+      <c r="M14" s="66"/>
       <c r="N14" s="29"/>
     </row>
     <row r="15" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="54"/>
-      <c r="L15" s="54"/>
-      <c r="M15" s="55"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="65"/>
+      <c r="E15" s="65"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
+      <c r="I15" s="65"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="65"/>
+      <c r="M15" s="66"/>
       <c r="N15" s="29"/>
     </row>
     <row r="16" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="54"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="54"/>
-      <c r="K16" s="54"/>
-      <c r="L16" s="54"/>
-      <c r="M16" s="55"/>
+      <c r="C16" s="65"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="65"/>
+      <c r="F16" s="65"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
+      <c r="I16" s="65"/>
+      <c r="J16" s="65"/>
+      <c r="K16" s="65"/>
+      <c r="L16" s="65"/>
+      <c r="M16" s="66"/>
       <c r="N16" s="29"/>
     </row>
     <row r="17" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="64" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54"/>
-      <c r="I17" s="54"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="54"/>
-      <c r="L17" s="54"/>
-      <c r="M17" s="55"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="65"/>
+      <c r="F17" s="65"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="65"/>
+      <c r="I17" s="65"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="65"/>
+      <c r="L17" s="65"/>
+      <c r="M17" s="66"/>
       <c r="N17" s="29"/>
     </row>
     <row r="18" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B18" s="53" t="s">
+      <c r="B18" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
-      <c r="J18" s="54"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="54"/>
-      <c r="M18" s="55"/>
+      <c r="C18" s="65"/>
+      <c r="D18" s="65"/>
+      <c r="E18" s="65"/>
+      <c r="F18" s="65"/>
+      <c r="G18" s="65"/>
+      <c r="H18" s="65"/>
+      <c r="I18" s="65"/>
+      <c r="J18" s="65"/>
+      <c r="K18" s="65"/>
+      <c r="L18" s="65"/>
+      <c r="M18" s="66"/>
       <c r="N18" s="29"/>
     </row>
     <row r="19" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B19" s="53" t="s">
+      <c r="B19" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="54"/>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
-      <c r="H19" s="54"/>
-      <c r="I19" s="54"/>
-      <c r="J19" s="54"/>
-      <c r="K19" s="54"/>
-      <c r="L19" s="54"/>
-      <c r="M19" s="55"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="65"/>
+      <c r="E19" s="65"/>
+      <c r="F19" s="65"/>
+      <c r="G19" s="65"/>
+      <c r="H19" s="65"/>
+      <c r="I19" s="65"/>
+      <c r="J19" s="65"/>
+      <c r="K19" s="65"/>
+      <c r="L19" s="65"/>
+      <c r="M19" s="66"/>
       <c r="N19" s="29"/>
     </row>
     <row r="20" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="67" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="57"/>
-      <c r="M20" s="58"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="68"/>
+      <c r="J20" s="68"/>
+      <c r="K20" s="68"/>
+      <c r="L20" s="68"/>
+      <c r="M20" s="69"/>
     </row>
     <row r="21" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B21" s="53" t="s">
+      <c r="B21" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="54"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
-      <c r="M21" s="55"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="65"/>
+      <c r="I21" s="65"/>
+      <c r="J21" s="65"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="65"/>
+      <c r="M21" s="66"/>
     </row>
     <row r="22" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B22" s="53" t="s">
+      <c r="B22" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="54"/>
-      <c r="J22" s="54"/>
-      <c r="K22" s="54"/>
-      <c r="L22" s="54"/>
-      <c r="M22" s="55"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="65"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="65"/>
+      <c r="I22" s="65"/>
+      <c r="J22" s="65"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="65"/>
+      <c r="M22" s="66"/>
     </row>
     <row r="23" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B23" s="53" t="s">
+      <c r="B23" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54"/>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54"/>
-      <c r="K23" s="54"/>
-      <c r="L23" s="54"/>
-      <c r="M23" s="55"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
+      <c r="H23" s="65"/>
+      <c r="I23" s="65"/>
+      <c r="J23" s="65"/>
+      <c r="K23" s="65"/>
+      <c r="L23" s="65"/>
+      <c r="M23" s="66"/>
     </row>
     <row r="24" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B24" s="53" t="s">
+      <c r="B24" s="64" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
-      <c r="G24" s="54"/>
-      <c r="H24" s="54"/>
-      <c r="I24" s="54"/>
-      <c r="J24" s="54"/>
-      <c r="K24" s="54"/>
-      <c r="L24" s="54"/>
-      <c r="M24" s="55"/>
+      <c r="C24" s="65"/>
+      <c r="D24" s="65"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="65"/>
+      <c r="G24" s="65"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
+      <c r="J24" s="65"/>
+      <c r="K24" s="65"/>
+      <c r="L24" s="65"/>
+      <c r="M24" s="66"/>
     </row>
     <row r="25" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B25" s="56" t="s">
+      <c r="B25" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="57"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="57"/>
-      <c r="J25" s="57"/>
-      <c r="K25" s="57"/>
-      <c r="L25" s="57"/>
-      <c r="M25" s="58"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="68"/>
+      <c r="E25" s="68"/>
+      <c r="F25" s="68"/>
+      <c r="G25" s="68"/>
+      <c r="H25" s="68"/>
+      <c r="I25" s="68"/>
+      <c r="J25" s="68"/>
+      <c r="K25" s="68"/>
+      <c r="L25" s="68"/>
+      <c r="M25" s="69"/>
     </row>
     <row r="26" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="64" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
-      <c r="I26" s="54"/>
-      <c r="J26" s="54"/>
-      <c r="K26" s="54"/>
-      <c r="L26" s="54"/>
-      <c r="M26" s="55"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+      <c r="I26" s="65"/>
+      <c r="J26" s="65"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="65"/>
+      <c r="M26" s="66"/>
     </row>
     <row r="27" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B27" s="53" t="s">
+      <c r="B27" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="54"/>
-      <c r="G27" s="54"/>
-      <c r="H27" s="54"/>
-      <c r="I27" s="54"/>
-      <c r="J27" s="54"/>
-      <c r="K27" s="54"/>
-      <c r="L27" s="54"/>
-      <c r="M27" s="55"/>
+      <c r="C27" s="65"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
+      <c r="I27" s="65"/>
+      <c r="J27" s="65"/>
+      <c r="K27" s="65"/>
+      <c r="L27" s="65"/>
+      <c r="M27" s="66"/>
     </row>
     <row r="28" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B28" s="53" t="s">
+      <c r="B28" s="64" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="54"/>
-      <c r="D28" s="54"/>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54"/>
-      <c r="G28" s="54"/>
-      <c r="H28" s="54"/>
-      <c r="I28" s="54"/>
-      <c r="J28" s="54"/>
-      <c r="K28" s="54"/>
-      <c r="L28" s="54"/>
-      <c r="M28" s="55"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="65"/>
+      <c r="I28" s="65"/>
+      <c r="J28" s="65"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="65"/>
+      <c r="M28" s="66"/>
     </row>
     <row r="29" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B29" s="53" t="s">
+      <c r="B29" s="64" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="54"/>
-      <c r="F29" s="54"/>
-      <c r="G29" s="54"/>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54"/>
-      <c r="K29" s="54"/>
-      <c r="L29" s="54"/>
-      <c r="M29" s="55"/>
+      <c r="C29" s="65"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="65"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+      <c r="I29" s="65"/>
+      <c r="J29" s="65"/>
+      <c r="K29" s="65"/>
+      <c r="L29" s="65"/>
+      <c r="M29" s="66"/>
     </row>
     <row r="30" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B30" s="56" t="s">
+      <c r="B30" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="57"/>
-      <c r="D30" s="57"/>
-      <c r="E30" s="57"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="57"/>
-      <c r="H30" s="57"/>
-      <c r="I30" s="57"/>
-      <c r="J30" s="57"/>
-      <c r="K30" s="57"/>
-      <c r="L30" s="57"/>
-      <c r="M30" s="58"/>
+      <c r="C30" s="68"/>
+      <c r="D30" s="68"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="68"/>
+      <c r="I30" s="68"/>
+      <c r="J30" s="68"/>
+      <c r="K30" s="68"/>
+      <c r="L30" s="68"/>
+      <c r="M30" s="69"/>
     </row>
     <row r="31" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B31" s="53" t="s">
+      <c r="B31" s="64" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="54"/>
-      <c r="H31" s="54"/>
-      <c r="I31" s="54"/>
-      <c r="J31" s="54"/>
-      <c r="K31" s="54"/>
-      <c r="L31" s="54"/>
-      <c r="M31" s="55"/>
+      <c r="C31" s="65"/>
+      <c r="D31" s="65"/>
+      <c r="E31" s="65"/>
+      <c r="F31" s="65"/>
+      <c r="G31" s="65"/>
+      <c r="H31" s="65"/>
+      <c r="I31" s="65"/>
+      <c r="J31" s="65"/>
+      <c r="K31" s="65"/>
+      <c r="L31" s="65"/>
+      <c r="M31" s="66"/>
     </row>
     <row r="32" spans="2:14" ht="15" x14ac:dyDescent="0.2">
-      <c r="B32" s="53" t="s">
+      <c r="B32" s="64" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="54"/>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="54"/>
-      <c r="G32" s="54"/>
-      <c r="H32" s="54"/>
-      <c r="I32" s="54"/>
-      <c r="J32" s="54"/>
-      <c r="K32" s="54"/>
-      <c r="L32" s="54"/>
-      <c r="M32" s="55"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="65"/>
+      <c r="G32" s="65"/>
+      <c r="H32" s="65"/>
+      <c r="I32" s="65"/>
+      <c r="J32" s="65"/>
+      <c r="K32" s="65"/>
+      <c r="L32" s="65"/>
+      <c r="M32" s="66"/>
     </row>
     <row r="33" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B33" s="56" t="s">
+      <c r="B33" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="57"/>
-      <c r="D33" s="57"/>
-      <c r="E33" s="57"/>
-      <c r="F33" s="57"/>
-      <c r="G33" s="57"/>
-      <c r="H33" s="57"/>
-      <c r="I33" s="57"/>
-      <c r="J33" s="57"/>
-      <c r="K33" s="57"/>
-      <c r="L33" s="57"/>
-      <c r="M33" s="58"/>
+      <c r="C33" s="68"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="68"/>
+      <c r="F33" s="68"/>
+      <c r="G33" s="68"/>
+      <c r="H33" s="68"/>
+      <c r="I33" s="68"/>
+      <c r="J33" s="68"/>
+      <c r="K33" s="68"/>
+      <c r="L33" s="68"/>
+      <c r="M33" s="69"/>
     </row>
     <row r="34" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B34" s="53" t="s">
+      <c r="B34" s="64" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="54"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="54"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="54"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="54"/>
-      <c r="K34" s="54"/>
-      <c r="L34" s="54"/>
-      <c r="M34" s="55"/>
+      <c r="C34" s="65"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="65"/>
+      <c r="G34" s="65"/>
+      <c r="H34" s="65"/>
+      <c r="I34" s="65"/>
+      <c r="J34" s="65"/>
+      <c r="K34" s="65"/>
+      <c r="L34" s="65"/>
+      <c r="M34" s="66"/>
     </row>
     <row r="35" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="54"/>
-      <c r="G35" s="54"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="54"/>
-      <c r="J35" s="54"/>
-      <c r="K35" s="54"/>
-      <c r="L35" s="54"/>
-      <c r="M35" s="55"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
+      <c r="K35" s="65"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="66"/>
     </row>
     <row r="36" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B36" s="56" t="s">
+      <c r="B36" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="C36" s="57"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="57"/>
-      <c r="F36" s="57"/>
-      <c r="G36" s="57"/>
-      <c r="H36" s="57"/>
-      <c r="I36" s="57"/>
-      <c r="J36" s="57"/>
-      <c r="K36" s="57"/>
-      <c r="L36" s="57"/>
-      <c r="M36" s="58"/>
+      <c r="C36" s="68"/>
+      <c r="D36" s="68"/>
+      <c r="E36" s="68"/>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+      <c r="I36" s="68"/>
+      <c r="J36" s="68"/>
+      <c r="K36" s="68"/>
+      <c r="L36" s="68"/>
+      <c r="M36" s="69"/>
     </row>
     <row r="37" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B37" s="53" t="s">
+      <c r="B37" s="64" t="s">
         <v>82</v>
       </c>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="54"/>
-      <c r="H37" s="54"/>
-      <c r="I37" s="54"/>
-      <c r="J37" s="54"/>
-      <c r="K37" s="54"/>
-      <c r="L37" s="54"/>
-      <c r="M37" s="55"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="65"/>
+      <c r="K37" s="65"/>
+      <c r="L37" s="65"/>
+      <c r="M37" s="66"/>
     </row>
     <row r="38" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="64" t="s">
         <v>83</v>
       </c>
-      <c r="C38" s="54"/>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="54"/>
-      <c r="H38" s="54"/>
-      <c r="I38" s="54"/>
-      <c r="J38" s="54"/>
-      <c r="K38" s="54"/>
-      <c r="L38" s="54"/>
-      <c r="M38" s="55"/>
+      <c r="C38" s="65"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="65"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="65"/>
+      <c r="J38" s="65"/>
+      <c r="K38" s="65"/>
+      <c r="L38" s="65"/>
+      <c r="M38" s="66"/>
     </row>
     <row r="39" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B39" s="53" t="s">
+      <c r="B39" s="64" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="54"/>
-      <c r="F39" s="54"/>
-      <c r="G39" s="54"/>
-      <c r="H39" s="54"/>
-      <c r="I39" s="54"/>
-      <c r="J39" s="54"/>
-      <c r="K39" s="54"/>
-      <c r="L39" s="54"/>
-      <c r="M39" s="55"/>
+      <c r="C39" s="65"/>
+      <c r="D39" s="65"/>
+      <c r="E39" s="65"/>
+      <c r="F39" s="65"/>
+      <c r="G39" s="65"/>
+      <c r="H39" s="65"/>
+      <c r="I39" s="65"/>
+      <c r="J39" s="65"/>
+      <c r="K39" s="65"/>
+      <c r="L39" s="65"/>
+      <c r="M39" s="66"/>
     </row>
     <row r="40" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B40" s="53" t="s">
+      <c r="B40" s="64" t="s">
         <v>85</v>
       </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="54"/>
-      <c r="G40" s="54"/>
-      <c r="H40" s="54"/>
-      <c r="I40" s="54"/>
-      <c r="J40" s="54"/>
-      <c r="K40" s="54"/>
-      <c r="L40" s="54"/>
-      <c r="M40" s="55"/>
+      <c r="C40" s="65"/>
+      <c r="D40" s="65"/>
+      <c r="E40" s="65"/>
+      <c r="F40" s="65"/>
+      <c r="G40" s="65"/>
+      <c r="H40" s="65"/>
+      <c r="I40" s="65"/>
+      <c r="J40" s="65"/>
+      <c r="K40" s="65"/>
+      <c r="L40" s="65"/>
+      <c r="M40" s="66"/>
     </row>
     <row r="41" spans="2:13" ht="18" x14ac:dyDescent="0.2">
-      <c r="B41" s="59" t="s">
+      <c r="B41" s="70" t="s">
         <v>113</v>
       </c>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="60"/>
-      <c r="G41" s="60"/>
-      <c r="H41" s="60"/>
-      <c r="I41" s="60"/>
-      <c r="J41" s="60"/>
-      <c r="K41" s="60"/>
-      <c r="L41" s="60"/>
-      <c r="M41" s="61"/>
+      <c r="C41" s="71"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="71"/>
+      <c r="F41" s="71"/>
+      <c r="G41" s="71"/>
+      <c r="H41" s="71"/>
+      <c r="I41" s="71"/>
+      <c r="J41" s="71"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
+      <c r="M41" s="72"/>
     </row>
     <row r="42" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B42" s="53" t="s">
+      <c r="B42" s="64" t="s">
         <v>86</v>
       </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54"/>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54"/>
-      <c r="K42" s="54"/>
-      <c r="L42" s="54"/>
-      <c r="M42" s="55"/>
+      <c r="C42" s="65"/>
+      <c r="D42" s="65"/>
+      <c r="E42" s="65"/>
+      <c r="F42" s="65"/>
+      <c r="G42" s="65"/>
+      <c r="H42" s="65"/>
+      <c r="I42" s="65"/>
+      <c r="J42" s="65"/>
+      <c r="K42" s="65"/>
+      <c r="L42" s="65"/>
+      <c r="M42" s="66"/>
     </row>
     <row r="43" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B43" s="53" t="s">
+      <c r="B43" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="C43" s="54"/>
-      <c r="D43" s="54"/>
-      <c r="E43" s="54"/>
-      <c r="F43" s="54"/>
-      <c r="G43" s="54"/>
-      <c r="H43" s="54"/>
-      <c r="I43" s="54"/>
-      <c r="J43" s="54"/>
-      <c r="K43" s="54"/>
-      <c r="L43" s="54"/>
-      <c r="M43" s="55"/>
+      <c r="C43" s="65"/>
+      <c r="D43" s="65"/>
+      <c r="E43" s="65"/>
+      <c r="F43" s="65"/>
+      <c r="G43" s="65"/>
+      <c r="H43" s="65"/>
+      <c r="I43" s="65"/>
+      <c r="J43" s="65"/>
+      <c r="K43" s="65"/>
+      <c r="L43" s="65"/>
+      <c r="M43" s="66"/>
     </row>
     <row r="44" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B44" s="53" t="s">
+      <c r="B44" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="54"/>
-      <c r="D44" s="54"/>
-      <c r="E44" s="54"/>
-      <c r="F44" s="54"/>
-      <c r="G44" s="54"/>
-      <c r="H44" s="54"/>
-      <c r="I44" s="54"/>
-      <c r="J44" s="54"/>
-      <c r="K44" s="54"/>
-      <c r="L44" s="54"/>
-      <c r="M44" s="55"/>
+      <c r="C44" s="65"/>
+      <c r="D44" s="65"/>
+      <c r="E44" s="65"/>
+      <c r="F44" s="65"/>
+      <c r="G44" s="65"/>
+      <c r="H44" s="65"/>
+      <c r="I44" s="65"/>
+      <c r="J44" s="65"/>
+      <c r="K44" s="65"/>
+      <c r="L44" s="65"/>
+      <c r="M44" s="66"/>
     </row>
     <row r="45" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B45" s="53" t="s">
+      <c r="B45" s="64" t="s">
         <v>89</v>
       </c>
-      <c r="C45" s="54"/>
-      <c r="D45" s="54"/>
-      <c r="E45" s="54"/>
-      <c r="F45" s="54"/>
-      <c r="G45" s="54"/>
-      <c r="H45" s="54"/>
-      <c r="I45" s="54"/>
-      <c r="J45" s="54"/>
-      <c r="K45" s="54"/>
-      <c r="L45" s="54"/>
-      <c r="M45" s="55"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="65"/>
+      <c r="E45" s="65"/>
+      <c r="F45" s="65"/>
+      <c r="G45" s="65"/>
+      <c r="H45" s="65"/>
+      <c r="I45" s="65"/>
+      <c r="J45" s="65"/>
+      <c r="K45" s="65"/>
+      <c r="L45" s="65"/>
+      <c r="M45" s="66"/>
     </row>
     <row r="46" spans="2:13" ht="18" x14ac:dyDescent="0.2">
-      <c r="B46" s="59" t="s">
+      <c r="B46" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="C46" s="60"/>
-      <c r="D46" s="60"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="60"/>
-      <c r="G46" s="60"/>
-      <c r="H46" s="60"/>
-      <c r="I46" s="60"/>
-      <c r="J46" s="60"/>
-      <c r="K46" s="60"/>
-      <c r="L46" s="60"/>
-      <c r="M46" s="61"/>
+      <c r="C46" s="71"/>
+      <c r="D46" s="71"/>
+      <c r="E46" s="71"/>
+      <c r="F46" s="71"/>
+      <c r="G46" s="71"/>
+      <c r="H46" s="71"/>
+      <c r="I46" s="71"/>
+      <c r="J46" s="71"/>
+      <c r="K46" s="71"/>
+      <c r="L46" s="71"/>
+      <c r="M46" s="72"/>
     </row>
     <row r="47" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B47" s="53" t="s">
+      <c r="B47" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="54"/>
-      <c r="H47" s="54"/>
-      <c r="I47" s="54"/>
-      <c r="J47" s="54"/>
-      <c r="K47" s="54"/>
-      <c r="L47" s="54"/>
-      <c r="M47" s="55"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="65"/>
+      <c r="E47" s="65"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="65"/>
+      <c r="I47" s="65"/>
+      <c r="J47" s="65"/>
+      <c r="K47" s="65"/>
+      <c r="L47" s="65"/>
+      <c r="M47" s="66"/>
     </row>
     <row r="48" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B48" s="53" t="s">
+      <c r="B48" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="C48" s="54"/>
-      <c r="D48" s="54"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="54"/>
-      <c r="G48" s="54"/>
-      <c r="H48" s="54"/>
-      <c r="I48" s="54"/>
-      <c r="J48" s="54"/>
-      <c r="K48" s="54"/>
-      <c r="L48" s="54"/>
-      <c r="M48" s="55"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="65"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="65"/>
+      <c r="G48" s="65"/>
+      <c r="H48" s="65"/>
+      <c r="I48" s="65"/>
+      <c r="J48" s="65"/>
+      <c r="K48" s="65"/>
+      <c r="L48" s="65"/>
+      <c r="M48" s="66"/>
     </row>
     <row r="49" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B49" s="53" t="s">
+      <c r="B49" s="64" t="s">
         <v>92</v>
       </c>
-      <c r="C49" s="54"/>
-      <c r="D49" s="54"/>
-      <c r="E49" s="54"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="54"/>
-      <c r="H49" s="54"/>
-      <c r="I49" s="54"/>
-      <c r="J49" s="54"/>
-      <c r="K49" s="54"/>
-      <c r="L49" s="54"/>
-      <c r="M49" s="55"/>
+      <c r="C49" s="65"/>
+      <c r="D49" s="65"/>
+      <c r="E49" s="65"/>
+      <c r="F49" s="65"/>
+      <c r="G49" s="65"/>
+      <c r="H49" s="65"/>
+      <c r="I49" s="65"/>
+      <c r="J49" s="65"/>
+      <c r="K49" s="65"/>
+      <c r="L49" s="65"/>
+      <c r="M49" s="66"/>
     </row>
     <row r="50" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B50" s="53" t="s">
+      <c r="B50" s="64" t="s">
         <v>93</v>
       </c>
-      <c r="C50" s="54"/>
-      <c r="D50" s="54"/>
-      <c r="E50" s="54"/>
-      <c r="F50" s="54"/>
-      <c r="G50" s="54"/>
-      <c r="H50" s="54"/>
-      <c r="I50" s="54"/>
-      <c r="J50" s="54"/>
-      <c r="K50" s="54"/>
-      <c r="L50" s="54"/>
-      <c r="M50" s="55"/>
+      <c r="C50" s="65"/>
+      <c r="D50" s="65"/>
+      <c r="E50" s="65"/>
+      <c r="F50" s="65"/>
+      <c r="G50" s="65"/>
+      <c r="H50" s="65"/>
+      <c r="I50" s="65"/>
+      <c r="J50" s="65"/>
+      <c r="K50" s="65"/>
+      <c r="L50" s="65"/>
+      <c r="M50" s="66"/>
     </row>
     <row r="51" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B51" s="53" t="s">
+      <c r="B51" s="64" t="s">
         <v>94</v>
       </c>
-      <c r="C51" s="54"/>
-      <c r="D51" s="54"/>
-      <c r="E51" s="54"/>
-      <c r="F51" s="54"/>
-      <c r="G51" s="54"/>
-      <c r="H51" s="54"/>
-      <c r="I51" s="54"/>
-      <c r="J51" s="54"/>
-      <c r="K51" s="54"/>
-      <c r="L51" s="54"/>
-      <c r="M51" s="55"/>
+      <c r="C51" s="65"/>
+      <c r="D51" s="65"/>
+      <c r="E51" s="65"/>
+      <c r="F51" s="65"/>
+      <c r="G51" s="65"/>
+      <c r="H51" s="65"/>
+      <c r="I51" s="65"/>
+      <c r="J51" s="65"/>
+      <c r="K51" s="65"/>
+      <c r="L51" s="65"/>
+      <c r="M51" s="66"/>
     </row>
     <row r="52" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B52" s="53" t="s">
+      <c r="B52" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="C52" s="54"/>
-      <c r="D52" s="54"/>
-      <c r="E52" s="54"/>
-      <c r="F52" s="54"/>
-      <c r="G52" s="54"/>
-      <c r="H52" s="54"/>
-      <c r="I52" s="54"/>
-      <c r="J52" s="54"/>
-      <c r="K52" s="54"/>
-      <c r="L52" s="54"/>
-      <c r="M52" s="55"/>
+      <c r="C52" s="65"/>
+      <c r="D52" s="65"/>
+      <c r="E52" s="65"/>
+      <c r="F52" s="65"/>
+      <c r="G52" s="65"/>
+      <c r="H52" s="65"/>
+      <c r="I52" s="65"/>
+      <c r="J52" s="65"/>
+      <c r="K52" s="65"/>
+      <c r="L52" s="65"/>
+      <c r="M52" s="66"/>
     </row>
     <row r="53" spans="2:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="B53" s="68" t="s">
+      <c r="B53" s="79" t="s">
         <v>96</v>
       </c>
-      <c r="C53" s="69"/>
-      <c r="D53" s="69"/>
-      <c r="E53" s="69"/>
-      <c r="F53" s="69"/>
-      <c r="G53" s="69"/>
-      <c r="H53" s="69"/>
-      <c r="I53" s="69"/>
-      <c r="J53" s="69"/>
-      <c r="K53" s="69"/>
-      <c r="L53" s="69"/>
-      <c r="M53" s="70"/>
+      <c r="C53" s="80"/>
+      <c r="D53" s="80"/>
+      <c r="E53" s="80"/>
+      <c r="F53" s="80"/>
+      <c r="G53" s="80"/>
+      <c r="H53" s="80"/>
+      <c r="I53" s="80"/>
+      <c r="J53" s="80"/>
+      <c r="K53" s="80"/>
+      <c r="L53" s="80"/>
+      <c r="M53" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="51">
@@ -2351,14 +2392,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
@@ -2504,6 +2545,9 @@
         <v>22</v>
       </c>
       <c r="D5" s="18"/>
+      <c r="F5" s="58" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="25">
@@ -2512,8 +2556,11 @@
       <c r="C6" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="78">
-        <v>2</v>
+      <c r="D6" s="54">
+        <v>2</v>
+      </c>
+      <c r="F6" s="59" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2524,8 +2571,11 @@
       <c r="C7" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="77">
-        <v>2</v>
+      <c r="D7" s="53">
+        <v>2</v>
+      </c>
+      <c r="F7" s="60" t="s">
+        <v>98</v>
       </c>
       <c r="H7" s="11"/>
     </row>
@@ -2537,7 +2587,7 @@
       <c r="C8" s="45" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="77">
+      <c r="D8" s="53">
         <v>2</v>
       </c>
       <c r="H8" s="11"/>
@@ -2550,7 +2600,7 @@
       <c r="C9" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="77">
+      <c r="D9" s="53">
         <v>2</v>
       </c>
       <c r="H9" s="11"/>
@@ -2563,7 +2613,7 @@
       <c r="C10" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="55">
         <v>2</v>
       </c>
       <c r="H10" s="11"/>
@@ -2576,7 +2626,7 @@
       <c r="C11" s="45" t="s">
         <v>125</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="55">
         <v>2</v>
       </c>
       <c r="H11" s="11"/>
@@ -2589,7 +2639,7 @@
       <c r="C12" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="55">
         <v>2</v>
       </c>
       <c r="H12" s="11"/>
@@ -2602,7 +2652,7 @@
       <c r="C13" s="45" t="s">
         <v>128</v>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="55">
         <v>3</v>
       </c>
       <c r="H13" s="11"/>
@@ -2615,7 +2665,7 @@
       <c r="C14" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="77">
+      <c r="D14" s="53">
         <v>2</v>
       </c>
     </row>
@@ -2627,7 +2677,7 @@
       <c r="C15" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="77">
+      <c r="D15" s="53">
         <v>4</v>
       </c>
     </row>
@@ -2639,7 +2689,7 @@
       <c r="C16" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="77">
+      <c r="D16" s="53">
         <v>2</v>
       </c>
     </row>
@@ -2663,7 +2713,7 @@
       <c r="C18" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="55">
         <v>2</v>
       </c>
     </row>
@@ -2699,7 +2749,7 @@
       <c r="C21" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="38">
+      <c r="D21" s="57">
         <v>2</v>
       </c>
     </row>
@@ -2711,7 +2761,7 @@
       <c r="C22" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="61">
         <v>2</v>
       </c>
     </row>
@@ -2765,7 +2815,7 @@
       <c r="C27" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="38">
+      <c r="D27" s="55">
         <v>3</v>
       </c>
     </row>
@@ -2777,7 +2827,7 @@
       <c r="C28" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D28" s="38">
+      <c r="D28" s="55">
         <v>1</v>
       </c>
     </row>
@@ -2789,7 +2839,7 @@
       <c r="C29" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D29" s="55">
         <v>3</v>
       </c>
     </row>
@@ -2843,7 +2893,7 @@
       <c r="C34" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D34" s="38">
+      <c r="D34" s="57">
         <v>3</v>
       </c>
     </row>
@@ -2855,7 +2905,7 @@
       <c r="C35" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="D35" s="38">
+      <c r="D35" s="57">
         <v>2</v>
       </c>
     </row>
@@ -3027,7 +3077,7 @@
     <col min="3" max="3" width="7.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.42578125" customWidth="1"/>
     <col min="8" max="8" width="13.42578125" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
@@ -3035,18 +3085,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
@@ -3060,10 +3110,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" s="5"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
@@ -3113,18 +3163,18 @@
       <c r="J5" s="4"/>
     </row>
     <row r="6" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73"/>
-      <c r="H6" s="73"/>
-      <c r="I6" s="74"/>
-      <c r="J6" s="73"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="84"/>
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="84"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="31">
@@ -3139,16 +3189,16 @@
       <c r="D7" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="44" t="s">
+      <c r="E7" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="62" t="s">
         <v>132</v>
       </c>
-      <c r="H7" s="79" t="s">
+      <c r="H7" s="63" t="s">
         <v>132</v>
       </c>
       <c r="I7" s="4">
@@ -3169,16 +3219,16 @@
       <c r="D8" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="62" t="s">
         <v>132</v>
       </c>
-      <c r="H8" s="79" t="s">
+      <c r="H8" s="63" t="s">
         <v>133</v>
       </c>
       <c r="I8" s="4">
@@ -3199,16 +3249,16 @@
       <c r="D9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="E9" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="62" t="s">
         <v>135</v>
       </c>
-      <c r="H9" s="79" t="s">
+      <c r="H9" s="63" t="s">
         <v>135</v>
       </c>
       <c r="I9" s="4">
@@ -3229,16 +3279,16 @@
       <c r="D10" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="H10" s="79" t="s">
+      <c r="H10" s="63" t="s">
         <v>134</v>
       </c>
       <c r="I10" s="4">
@@ -3259,16 +3309,16 @@
       <c r="D11" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E11" s="44" t="s">
+      <c r="E11" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="62" t="s">
         <v>135</v>
       </c>
-      <c r="H11" s="79" t="s">
+      <c r="H11" s="63" t="s">
         <v>131</v>
       </c>
       <c r="I11" s="4">
@@ -3289,16 +3339,16 @@
       <c r="D12" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E12" s="44" t="s">
+      <c r="E12" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="H12" s="79" t="s">
+      <c r="H12" s="63" t="s">
         <v>134</v>
       </c>
       <c r="I12" s="4">
@@ -3319,16 +3369,16 @@
       <c r="D13" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E13" s="44" t="s">
+      <c r="E13" s="56" t="s">
         <v>130</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="H13" s="79" t="s">
+      <c r="H13" s="63" t="s">
         <v>135</v>
       </c>
       <c r="I13" s="4">
@@ -3337,16 +3387,16 @@
       <c r="J13" s="48"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="72"/>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
-      <c r="G14" s="72"/>
-      <c r="H14" s="72"/>
-      <c r="I14" s="72"/>
-      <c r="J14" s="72"/>
+      <c r="A14" s="83"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="83"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
+      <c r="J14" s="83"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="30" t="s">
@@ -3396,18 +3446,18 @@
       <c r="J19" s="4"/>
     </row>
     <row r="20" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="73" t="s">
+      <c r="A20" s="84" t="s">
         <v>97</v>
       </c>
-      <c r="B20" s="73"/>
-      <c r="C20" s="74"/>
-      <c r="D20" s="73"/>
-      <c r="E20" s="73"/>
-      <c r="F20" s="73"/>
-      <c r="G20" s="73"/>
-      <c r="H20" s="73"/>
-      <c r="I20" s="73"/>
-      <c r="J20" s="73"/>
+      <c r="B20" s="84"/>
+      <c r="C20" s="85"/>
+      <c r="D20" s="84"/>
+      <c r="E20" s="84"/>
+      <c r="F20" s="84"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="84"/>
+      <c r="I20" s="84"/>
+      <c r="J20" s="84"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="31">
@@ -3422,11 +3472,21 @@
       <c r="D21" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="4"/>
+      <c r="E21" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F21" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G21" s="62">
+        <v>45818</v>
+      </c>
+      <c r="H21" s="62">
+        <v>45818</v>
+      </c>
+      <c r="I21" s="4">
+        <v>2</v>
+      </c>
       <c r="J21" s="4"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -3442,11 +3502,21 @@
       <c r="D22" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="4"/>
+      <c r="E22" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F22" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G22" s="62">
+        <v>45910</v>
+      </c>
+      <c r="H22" s="62">
+        <v>45940</v>
+      </c>
+      <c r="I22" s="4">
+        <v>3</v>
+      </c>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -3462,11 +3532,21 @@
       <c r="D23" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="4"/>
+      <c r="E23" s="56" t="s">
+        <v>136</v>
+      </c>
+      <c r="F23" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G23" s="62">
+        <v>45879</v>
+      </c>
+      <c r="H23" s="62">
+        <v>45910</v>
+      </c>
+      <c r="I23" s="4">
+        <v>1</v>
+      </c>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -3482,11 +3562,21 @@
       <c r="D24" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="4"/>
+      <c r="E24" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F24" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G24" s="62">
+        <v>45818</v>
+      </c>
+      <c r="H24" s="62">
+        <v>45879</v>
+      </c>
+      <c r="I24" s="4">
+        <v>3</v>
+      </c>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -3502,11 +3592,21 @@
       <c r="D25" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="4"/>
+      <c r="E25" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F25" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G25" s="62">
+        <v>45757</v>
+      </c>
+      <c r="H25" s="62">
+        <v>45757</v>
+      </c>
+      <c r="I25" s="4">
+        <v>2</v>
+      </c>
       <c r="J25" s="4"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -3522,11 +3622,21 @@
       <c r="D26" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="4"/>
+      <c r="E26" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F26" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G26" s="62">
+        <v>45757</v>
+      </c>
+      <c r="H26" s="62">
+        <v>45787</v>
+      </c>
+      <c r="I26" s="4">
+        <v>2</v>
+      </c>
       <c r="J26" s="4"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
@@ -3542,11 +3652,21 @@
       <c r="D27" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="4"/>
+      <c r="E27" s="56" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G27" s="62">
+        <v>45787</v>
+      </c>
+      <c r="H27" s="62">
+        <v>45787</v>
+      </c>
+      <c r="I27" s="4">
+        <v>2</v>
+      </c>
       <c r="J27" s="4"/>
     </row>
     <row r="28" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -3562,24 +3682,34 @@
       <c r="D28" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="4"/>
+      <c r="E28" s="56">
+        <v>45757</v>
+      </c>
+      <c r="F28" s="62">
+        <v>45940</v>
+      </c>
+      <c r="G28" s="62">
+        <v>45787</v>
+      </c>
+      <c r="H28" s="62">
+        <v>45818</v>
+      </c>
+      <c r="I28" s="4">
+        <v>3</v>
+      </c>
       <c r="J28" s="4"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="72"/>
-      <c r="B29" s="72"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="72"/>
-      <c r="E29" s="72"/>
-      <c r="F29" s="72"/>
-      <c r="G29" s="72"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="72"/>
-      <c r="J29" s="72"/>
+      <c r="A29" s="83"/>
+      <c r="B29" s="83"/>
+      <c r="C29" s="86"/>
+      <c r="D29" s="83"/>
+      <c r="E29" s="83"/>
+      <c r="F29" s="83"/>
+      <c r="G29" s="83"/>
+      <c r="H29" s="83"/>
+      <c r="I29" s="83"/>
+      <c r="J29" s="83"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="30" t="s">
@@ -3629,18 +3759,18 @@
       <c r="J34" s="4"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="73" t="s">
+      <c r="A35" s="84" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="73"/>
-      <c r="C35" s="73"/>
-      <c r="D35" s="73"/>
-      <c r="E35" s="73"/>
-      <c r="F35" s="73"/>
-      <c r="G35" s="73"/>
-      <c r="H35" s="73"/>
-      <c r="I35" s="73"/>
-      <c r="J35" s="73"/>
+      <c r="B35" s="84"/>
+      <c r="C35" s="84"/>
+      <c r="D35" s="84"/>
+      <c r="E35" s="84"/>
+      <c r="F35" s="84"/>
+      <c r="G35" s="84"/>
+      <c r="H35" s="84"/>
+      <c r="I35" s="84"/>
+      <c r="J35" s="84"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="31">
@@ -3655,11 +3785,21 @@
       <c r="D36" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="4"/>
+      <c r="E36" s="62">
+        <v>45940</v>
+      </c>
+      <c r="F36" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="G36" s="62">
+        <v>45971</v>
+      </c>
+      <c r="H36" s="62" t="s">
+        <v>138</v>
+      </c>
+      <c r="I36" s="4">
+        <v>3</v>
+      </c>
       <c r="J36" s="4"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
@@ -3675,11 +3815,21 @@
       <c r="D37" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="4"/>
+      <c r="E37" s="62">
+        <v>45940</v>
+      </c>
+      <c r="F37" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="G37" s="62" t="s">
+        <v>138</v>
+      </c>
+      <c r="H37" s="62" t="s">
+        <v>139</v>
+      </c>
+      <c r="I37" s="4">
+        <v>2</v>
+      </c>
       <c r="J37" s="4"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -3695,11 +3845,21 @@
       <c r="D38" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="4"/>
+      <c r="E38" s="62">
+        <v>45940</v>
+      </c>
+      <c r="F38" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="G38" s="62">
+        <v>45940</v>
+      </c>
+      <c r="H38" s="62">
+        <v>45940</v>
+      </c>
+      <c r="I38" s="4">
+        <v>2</v>
+      </c>
       <c r="J38" s="4"/>
     </row>
     <row r="39" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -3715,24 +3875,34 @@
       <c r="D39" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="4"/>
+      <c r="E39" s="62">
+        <v>45940</v>
+      </c>
+      <c r="F39" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="G39" s="62">
+        <v>45940</v>
+      </c>
+      <c r="H39" s="62">
+        <v>45971</v>
+      </c>
+      <c r="I39" s="4">
+        <v>2</v>
+      </c>
       <c r="J39" s="4"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A40" s="72"/>
-      <c r="B40" s="72"/>
-      <c r="C40" s="72"/>
-      <c r="D40" s="72"/>
-      <c r="E40" s="72"/>
-      <c r="F40" s="72"/>
-      <c r="G40" s="72"/>
-      <c r="H40" s="72"/>
-      <c r="I40" s="72"/>
-      <c r="J40" s="72"/>
+      <c r="A40" s="83"/>
+      <c r="B40" s="83"/>
+      <c r="C40" s="83"/>
+      <c r="D40" s="83"/>
+      <c r="E40" s="83"/>
+      <c r="F40" s="83"/>
+      <c r="G40" s="83"/>
+      <c r="H40" s="83"/>
+      <c r="I40" s="83"/>
+      <c r="J40" s="83"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="30" t="s">
@@ -3782,18 +3952,18 @@
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="73" t="s">
+      <c r="A46" s="84" t="s">
         <v>99</v>
       </c>
-      <c r="B46" s="73"/>
-      <c r="C46" s="73"/>
-      <c r="D46" s="73"/>
-      <c r="E46" s="73"/>
-      <c r="F46" s="73"/>
-      <c r="G46" s="73"/>
-      <c r="H46" s="73"/>
-      <c r="I46" s="73"/>
-      <c r="J46" s="73"/>
+      <c r="B46" s="84"/>
+      <c r="C46" s="84"/>
+      <c r="D46" s="84"/>
+      <c r="E46" s="84"/>
+      <c r="F46" s="84"/>
+      <c r="G46" s="84"/>
+      <c r="H46" s="84"/>
+      <c r="I46" s="84"/>
+      <c r="J46" s="84"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="31">
@@ -3808,8 +3978,12 @@
       <c r="D47" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
+      <c r="E47" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>140</v>
+      </c>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
       <c r="I47" s="4"/>
@@ -3828,8 +4002,12 @@
       <c r="D48" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
+      <c r="E48" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>140</v>
+      </c>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
       <c r="I48" s="4"/>
@@ -3848,24 +4026,28 @@
       <c r="D49" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
+      <c r="E49" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>140</v>
+      </c>
       <c r="G49" s="7"/>
       <c r="H49" s="7"/>
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" s="72"/>
-      <c r="B50" s="72"/>
-      <c r="C50" s="72"/>
-      <c r="D50" s="72"/>
-      <c r="E50" s="72"/>
-      <c r="F50" s="72"/>
-      <c r="G50" s="72"/>
-      <c r="H50" s="72"/>
-      <c r="I50" s="72"/>
-      <c r="J50" s="72"/>
+      <c r="A50" s="83"/>
+      <c r="B50" s="83"/>
+      <c r="C50" s="83"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
+      <c r="J50" s="83"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="30" t="s">
@@ -3915,18 +4097,18 @@
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="73" t="s">
+      <c r="A56" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="B56" s="74"/>
-      <c r="C56" s="74"/>
-      <c r="D56" s="73"/>
-      <c r="E56" s="73"/>
-      <c r="F56" s="73"/>
-      <c r="G56" s="73"/>
-      <c r="H56" s="73"/>
-      <c r="I56" s="73"/>
-      <c r="J56" s="73"/>
+      <c r="B56" s="85"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="84"/>
+      <c r="E56" s="84"/>
+      <c r="F56" s="84"/>
+      <c r="G56" s="84"/>
+      <c r="H56" s="84"/>
+      <c r="I56" s="84"/>
+      <c r="J56" s="84"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="49">
@@ -3989,16 +4171,16 @@
       <c r="J59" s="4"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" s="72"/>
-      <c r="B60" s="75"/>
-      <c r="C60" s="75"/>
-      <c r="D60" s="72"/>
-      <c r="E60" s="72"/>
-      <c r="F60" s="72"/>
-      <c r="G60" s="72"/>
-      <c r="H60" s="72"/>
-      <c r="I60" s="72"/>
-      <c r="J60" s="72"/>
+      <c r="A60" s="83"/>
+      <c r="B60" s="86"/>
+      <c r="C60" s="86"/>
+      <c r="D60" s="83"/>
+      <c r="E60" s="83"/>
+      <c r="F60" s="83"/>
+      <c r="G60" s="83"/>
+      <c r="H60" s="83"/>
+      <c r="I60" s="83"/>
+      <c r="J60" s="83"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="30" t="s">
@@ -4048,18 +4230,18 @@
       <c r="J65" s="4"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A66" s="73" t="s">
+      <c r="A66" s="84" t="s">
         <v>101</v>
       </c>
-      <c r="B66" s="73"/>
-      <c r="C66" s="73"/>
-      <c r="D66" s="73"/>
-      <c r="E66" s="73"/>
-      <c r="F66" s="73"/>
-      <c r="G66" s="73"/>
-      <c r="H66" s="73"/>
-      <c r="I66" s="73"/>
-      <c r="J66" s="73"/>
+      <c r="B66" s="84"/>
+      <c r="C66" s="84"/>
+      <c r="D66" s="84"/>
+      <c r="E66" s="84"/>
+      <c r="F66" s="84"/>
+      <c r="G66" s="84"/>
+      <c r="H66" s="84"/>
+      <c r="I66" s="84"/>
+      <c r="J66" s="84"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="31">
@@ -4102,16 +4284,16 @@
       <c r="J68" s="4"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A69" s="72"/>
-      <c r="B69" s="72"/>
-      <c r="C69" s="72"/>
-      <c r="D69" s="72"/>
-      <c r="E69" s="72"/>
-      <c r="F69" s="72"/>
-      <c r="G69" s="72"/>
-      <c r="H69" s="72"/>
-      <c r="I69" s="72"/>
-      <c r="J69" s="72"/>
+      <c r="A69" s="83"/>
+      <c r="B69" s="83"/>
+      <c r="C69" s="83"/>
+      <c r="D69" s="83"/>
+      <c r="E69" s="83"/>
+      <c r="F69" s="83"/>
+      <c r="G69" s="83"/>
+      <c r="H69" s="83"/>
+      <c r="I69" s="83"/>
+      <c r="J69" s="83"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="30" t="s">
@@ -4161,18 +4343,18 @@
       <c r="J74" s="4"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" s="73" t="s">
+      <c r="A75" s="84" t="s">
         <v>102</v>
       </c>
-      <c r="B75" s="73"/>
-      <c r="C75" s="73"/>
-      <c r="D75" s="73"/>
-      <c r="E75" s="73"/>
-      <c r="F75" s="73"/>
-      <c r="G75" s="73"/>
-      <c r="H75" s="73"/>
-      <c r="I75" s="73"/>
-      <c r="J75" s="73"/>
+      <c r="B75" s="84"/>
+      <c r="C75" s="84"/>
+      <c r="D75" s="84"/>
+      <c r="E75" s="84"/>
+      <c r="F75" s="84"/>
+      <c r="G75" s="84"/>
+      <c r="H75" s="84"/>
+      <c r="I75" s="84"/>
+      <c r="J75" s="84"/>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="31">
@@ -4215,16 +4397,16 @@
       <c r="J77" s="4"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A78" s="72"/>
-      <c r="B78" s="72"/>
-      <c r="C78" s="72"/>
-      <c r="D78" s="72"/>
-      <c r="E78" s="72"/>
-      <c r="F78" s="72"/>
-      <c r="G78" s="72"/>
-      <c r="H78" s="72"/>
-      <c r="I78" s="72"/>
-      <c r="J78" s="72"/>
+      <c r="A78" s="83"/>
+      <c r="B78" s="83"/>
+      <c r="C78" s="83"/>
+      <c r="D78" s="83"/>
+      <c r="E78" s="83"/>
+      <c r="F78" s="83"/>
+      <c r="G78" s="83"/>
+      <c r="H78" s="83"/>
+      <c r="I78" s="83"/>
+      <c r="J78" s="83"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="30" t="s">
@@ -4274,18 +4456,18 @@
       <c r="J83" s="4"/>
     </row>
     <row r="84" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="73" t="s">
+      <c r="A84" s="84" t="s">
         <v>103</v>
       </c>
-      <c r="B84" s="73"/>
-      <c r="C84" s="73"/>
-      <c r="D84" s="73"/>
-      <c r="E84" s="73"/>
-      <c r="F84" s="73"/>
-      <c r="G84" s="73"/>
-      <c r="H84" s="73"/>
-      <c r="I84" s="73"/>
-      <c r="J84" s="73"/>
+      <c r="B84" s="84"/>
+      <c r="C84" s="84"/>
+      <c r="D84" s="84"/>
+      <c r="E84" s="84"/>
+      <c r="F84" s="84"/>
+      <c r="G84" s="84"/>
+      <c r="H84" s="84"/>
+      <c r="I84" s="84"/>
+      <c r="J84" s="84"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="31">
@@ -4328,16 +4510,16 @@
       <c r="J86" s="4"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A87" s="72"/>
-      <c r="B87" s="72"/>
-      <c r="C87" s="72"/>
-      <c r="D87" s="72"/>
-      <c r="E87" s="72"/>
-      <c r="F87" s="72"/>
-      <c r="G87" s="72"/>
-      <c r="H87" s="72"/>
-      <c r="I87" s="72"/>
-      <c r="J87" s="72"/>
+      <c r="A87" s="83"/>
+      <c r="B87" s="83"/>
+      <c r="C87" s="83"/>
+      <c r="D87" s="83"/>
+      <c r="E87" s="83"/>
+      <c r="F87" s="83"/>
+      <c r="G87" s="83"/>
+      <c r="H87" s="83"/>
+      <c r="I87" s="83"/>
+      <c r="J87" s="83"/>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="30" t="s">
@@ -4387,18 +4569,18 @@
       <c r="J92" s="4"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A93" s="73" t="s">
+      <c r="A93" s="84" t="s">
         <v>104</v>
       </c>
-      <c r="B93" s="73"/>
-      <c r="C93" s="73"/>
-      <c r="D93" s="73"/>
-      <c r="E93" s="73"/>
-      <c r="F93" s="73"/>
-      <c r="G93" s="73"/>
-      <c r="H93" s="73"/>
-      <c r="I93" s="73"/>
-      <c r="J93" s="73"/>
+      <c r="B93" s="84"/>
+      <c r="C93" s="84"/>
+      <c r="D93" s="84"/>
+      <c r="E93" s="84"/>
+      <c r="F93" s="84"/>
+      <c r="G93" s="84"/>
+      <c r="H93" s="84"/>
+      <c r="I93" s="84"/>
+      <c r="J93" s="84"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="31">
@@ -4441,16 +4623,16 @@
       <c r="J95" s="4"/>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A96" s="72"/>
-      <c r="B96" s="72"/>
-      <c r="C96" s="72"/>
-      <c r="D96" s="72"/>
-      <c r="E96" s="72"/>
-      <c r="F96" s="72"/>
-      <c r="G96" s="72"/>
-      <c r="H96" s="72"/>
-      <c r="I96" s="72"/>
-      <c r="J96" s="72"/>
+      <c r="A96" s="83"/>
+      <c r="B96" s="83"/>
+      <c r="C96" s="83"/>
+      <c r="D96" s="83"/>
+      <c r="E96" s="83"/>
+      <c r="F96" s="83"/>
+      <c r="G96" s="83"/>
+      <c r="H96" s="83"/>
+      <c r="I96" s="83"/>
+      <c r="J96" s="83"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="30" t="s">
@@ -4500,18 +4682,18 @@
       <c r="J101" s="4"/>
     </row>
     <row r="102" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="73" t="s">
+      <c r="A102" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="B102" s="73"/>
-      <c r="C102" s="74"/>
-      <c r="D102" s="73"/>
-      <c r="E102" s="73"/>
-      <c r="F102" s="73"/>
-      <c r="G102" s="73"/>
-      <c r="H102" s="73"/>
-      <c r="I102" s="73"/>
-      <c r="J102" s="73"/>
+      <c r="B102" s="84"/>
+      <c r="C102" s="85"/>
+      <c r="D102" s="84"/>
+      <c r="E102" s="84"/>
+      <c r="F102" s="84"/>
+      <c r="G102" s="84"/>
+      <c r="H102" s="84"/>
+      <c r="I102" s="84"/>
+      <c r="J102" s="84"/>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" s="31">
@@ -4574,16 +4756,16 @@
       <c r="J105" s="4"/>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A106" s="72"/>
-      <c r="B106" s="72"/>
-      <c r="C106" s="75"/>
-      <c r="D106" s="72"/>
-      <c r="E106" s="72"/>
-      <c r="F106" s="72"/>
-      <c r="G106" s="72"/>
-      <c r="H106" s="72"/>
-      <c r="I106" s="72"/>
-      <c r="J106" s="72"/>
+      <c r="A106" s="83"/>
+      <c r="B106" s="83"/>
+      <c r="C106" s="86"/>
+      <c r="D106" s="83"/>
+      <c r="E106" s="83"/>
+      <c r="F106" s="83"/>
+      <c r="G106" s="83"/>
+      <c r="H106" s="83"/>
+      <c r="I106" s="83"/>
+      <c r="J106" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>